<commit_message>
Update(journal de travail C-H)
[10min] [DONE]

- Update du journal de travail personnel
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_MoserCharles-Henri.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_MoserCharles-Henri.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc01zcg\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1970BC24-C689-4768-91C5-50BFCF25255F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34B4FC5-0F0B-4C2A-9B99-C2D4A85DD9EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="61">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -203,6 +203,27 @@
   </si>
   <si>
     <t>Peer-Working Avec Antoine Piguet sur une erreur chez lui</t>
+  </si>
+  <si>
+    <t>Update de la page Details.vue pour que les étoiles s'affichent</t>
+  </si>
+  <si>
+    <t>Update du service API afin d'utiliser fetch à la place de Axios</t>
+  </si>
+  <si>
+    <t>Création de la page Mybooks, avec token d'authentification</t>
+  </si>
+  <si>
+    <t>Retravaillage de la page vue, pour que le header ne s'affiche pas sur le titre.</t>
+  </si>
+  <si>
+    <t>Creation de la page EditBooks + ajout de bouton pour modifier les données du livre que l'utilisateur à créer</t>
+  </si>
+  <si>
+    <t>Durant la journée, peer programming avec Antoine Piguet</t>
+  </si>
+  <si>
+    <t>update BooksView problème de routage.</t>
   </si>
 </sst>
 </file>
@@ -1133,13 +1154,13 @@
                   <c:v>2.0833333333333332E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.54513888888888884</c:v>
+                  <c:v>0.69444444444444442</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.0416666666666666E-2</c:v>
+                  <c:v>1.7361111111111112E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>6.5972222222222224E-2</c:v>
@@ -2111,7 +2132,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 16 heurs 34 minutes</v>
+        <v>0 jours 20 heurs 19 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2130,11 +2151,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>635</v>
+        <v>860</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>995</v>
+        <v>1220</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2727,107 +2748,173 @@
       <c r="G29" s="56"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="str">
+      <c r="A30" s="8">
         <f>IF(ISBLANK(B30),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B30))</f>
-        <v/>
-      </c>
-      <c r="B30" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B30" s="46">
+        <v>45797</v>
+      </c>
       <c r="C30" s="47"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="49"/>
-      <c r="F30" s="36"/>
+      <c r="D30" s="48">
+        <v>50</v>
+      </c>
+      <c r="E30" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="36" t="s">
+        <v>54</v>
+      </c>
       <c r="G30" s="55"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="str">
+      <c r="A31" s="16">
         <f>IF(ISBLANK(B31),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B31))</f>
-        <v/>
-      </c>
-      <c r="B31" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="B31" s="50">
+        <v>45797</v>
+      </c>
       <c r="C31" s="51"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="35"/>
+      <c r="D31" s="52">
+        <v>20</v>
+      </c>
+      <c r="E31" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="35" t="s">
+        <v>55</v>
+      </c>
       <c r="G31" s="56"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="str">
+      <c r="A32" s="8">
         <f>IF(ISBLANK(B32),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B32))</f>
-        <v/>
-      </c>
-      <c r="B32" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B32" s="46">
+        <v>45797</v>
+      </c>
       <c r="C32" s="47"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="36"/>
+      <c r="D32" s="48">
+        <v>50</v>
+      </c>
+      <c r="E32" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>56</v>
+      </c>
       <c r="G32" s="55"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="str">
+      <c r="A33" s="16">
         <f>IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
-        <v/>
-      </c>
-      <c r="B33" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="B33" s="50">
+        <v>45797</v>
+      </c>
       <c r="C33" s="51"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="35"/>
+      <c r="D33" s="52">
+        <v>5</v>
+      </c>
+      <c r="E33" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="35" t="s">
+        <v>57</v>
+      </c>
       <c r="G33" s="56"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="str">
+      <c r="A34" s="8">
         <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
-        <v/>
-      </c>
-      <c r="B34" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B34" s="46">
+        <v>45797</v>
+      </c>
       <c r="C34" s="47"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="35"/>
+      <c r="D34" s="48">
+        <v>40</v>
+      </c>
+      <c r="E34" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" s="35" t="s">
+        <v>58</v>
+      </c>
       <c r="G34" s="55"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="str">
+      <c r="A35" s="16">
         <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="B35" s="50">
+        <v>45797</v>
+      </c>
       <c r="C35" s="51"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="36"/>
+      <c r="D35" s="52">
+        <v>30</v>
+      </c>
+      <c r="E35" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" s="36" t="s">
+        <v>59</v>
+      </c>
       <c r="G35" s="56"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="str">
+      <c r="A36" s="8">
         <f>IF(ISBLANK(B36),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B36))</f>
-        <v/>
-      </c>
-      <c r="B36" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B36" s="46">
+        <v>45797</v>
+      </c>
       <c r="C36" s="47"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="35"/>
+      <c r="D36" s="48">
+        <v>20</v>
+      </c>
+      <c r="E36" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="35" t="s">
+        <v>60</v>
+      </c>
       <c r="G36" s="55"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="str">
+      <c r="A37" s="16">
         <f>IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
-        <v/>
-      </c>
-      <c r="B37" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="B37" s="50">
+        <v>45797</v>
+      </c>
       <c r="C37" s="51"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="35"/>
+      <c r="D37" s="52">
+        <v>10</v>
+      </c>
+      <c r="E37" s="53" t="s">
+        <v>6</v>
+      </c>
+      <c r="F37" s="35" t="s">
+        <v>0</v>
+      </c>
       <c r="G37" s="56"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="8" t="str">
+      <c r="A38" s="8">
         <f>IF(ISBLANK(B38),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B38))</f>
-        <v/>
-      </c>
-      <c r="B38" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B38" s="46">
+        <v>45798</v>
+      </c>
       <c r="C38" s="47"/>
       <c r="D38" s="48"/>
       <c r="E38" s="49"/>
@@ -2835,11 +2922,13 @@
       <c r="G38" s="55"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="str">
+      <c r="A39" s="16">
         <f>IF(ISBLANK(B39),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B39))</f>
-        <v/>
-      </c>
-      <c r="B39" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="B39" s="50">
+        <v>45798</v>
+      </c>
       <c r="C39" s="51"/>
       <c r="D39" s="52"/>
       <c r="E39" s="53"/>
@@ -2847,11 +2936,13 @@
       <c r="G39" s="56"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="str">
+      <c r="A40" s="8">
         <f>IF(ISBLANK(B40),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B40))</f>
-        <v/>
-      </c>
-      <c r="B40" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B40" s="46">
+        <v>45798</v>
+      </c>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="49"/>
@@ -8863,7 +8954,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>485</v>
+        <v>700</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8871,7 +8962,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.54513888888888884</v>
+        <v>0.69444444444444442</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8899,7 +8990,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -8907,7 +8998,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>1.0416666666666666E-2</v>
+        <v>1.7361111111111112E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -8988,7 +9079,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.69097222222222221</v>
+        <v>0.84722222222222232</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9011,6 +9102,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9233,17 +9335,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9253,6 +9344,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9269,15 +9371,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>